<commit_message>
update objet category instances
</commit_message>
<xml_diff>
--- a/objectCategories.xlsx
+++ b/objectCategories.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unigiessende-my.sharepoint.com/personal/gc2117_uni-giessen_de/Documents/Dokumente/GitHub/pep_wp4_eye_tracking/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="93" documentId="11_714DF4478877186C74FC37A4F8012D16618A742A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B22F034E-43B5-4E18-97A2-8B6107833B03}"/>
+  <xr:revisionPtr revIDLastSave="110" documentId="11_714DF4478877186C74FC37A4F8012D16618A742A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{11DB05D9-D175-4BD7-94C0-1DAE0BCE64C2}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="90" windowWidth="9780" windowHeight="10080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="683" uniqueCount="678">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="693">
   <si>
     <t>outlet</t>
   </si>
@@ -41,9 +41,6 @@
     <t>Category</t>
   </si>
   <si>
-    <t>animals</t>
-  </si>
-  <si>
     <t>apron</t>
   </si>
   <si>
@@ -2067,6 +2064,54 @@
   </si>
   <si>
     <t>glass wall/ shower</t>
+  </si>
+  <si>
+    <t>kettel</t>
+  </si>
+  <si>
+    <t>knif</t>
+  </si>
+  <si>
+    <t>light</t>
+  </si>
+  <si>
+    <t>person</t>
+  </si>
+  <si>
+    <t>animals/people</t>
+  </si>
+  <si>
+    <t>plants/flowers</t>
+  </si>
+  <si>
+    <t>shampoo holder</t>
+  </si>
+  <si>
+    <t>shower glass</t>
+  </si>
+  <si>
+    <t>shower head/shower</t>
+  </si>
+  <si>
+    <t>/shampoo</t>
+  </si>
+  <si>
+    <t>sticker</t>
+  </si>
+  <si>
+    <t>storage</t>
+  </si>
+  <si>
+    <t>sun</t>
+  </si>
+  <si>
+    <t>toarel hanger</t>
+  </si>
+  <si>
+    <t>towel/towel holder</t>
+  </si>
+  <si>
+    <t>wall mounted bidet</t>
   </si>
 </sst>
 </file>
@@ -2473,60 +2518,60 @@
         <v>1</v>
       </c>
       <c r="B1" t="s">
+        <v>155</v>
+      </c>
+      <c r="C1" t="s">
         <v>156</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>157</v>
       </c>
-      <c r="D1" t="s">
-        <v>158</v>
-      </c>
       <c r="E1" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F1" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="G1" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="H1" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="I1" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="J1" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="K1" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="L1" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="M1" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="N1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="O1" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="P1" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="Q1" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="R1" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>681</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -2535,18 +2580,21 @@
         <v>2</v>
       </c>
       <c r="D2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E2" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="F2" t="s">
-        <v>421</v>
+        <v>420</v>
+      </c>
+      <c r="G2" t="s">
+        <v>680</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -2555,12 +2603,12 @@
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -2569,12 +2617,12 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -2583,18 +2631,18 @@
         <v>8</v>
       </c>
       <c r="D5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E5" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="F5" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -2603,18 +2651,18 @@
         <v>9</v>
       </c>
       <c r="D6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E6" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="F6" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -2623,15 +2671,15 @@
         <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E7" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -2640,12 +2688,12 @@
         <v>0</v>
       </c>
       <c r="D8" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9">
         <v>16</v>
@@ -2654,21 +2702,21 @@
         <v>30</v>
       </c>
       <c r="D9" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E9" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="F9" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="G9" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B10">
         <v>82</v>
@@ -2677,18 +2725,18 @@
         <v>0</v>
       </c>
       <c r="D10" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E10" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F10" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B11">
         <v>2</v>
@@ -2697,12 +2745,12 @@
         <v>0</v>
       </c>
       <c r="D11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -2711,12 +2759,12 @@
         <v>1</v>
       </c>
       <c r="D12" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -2725,12 +2773,12 @@
         <v>1</v>
       </c>
       <c r="D13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B14">
         <v>6</v>
@@ -2739,18 +2787,21 @@
         <v>0</v>
       </c>
       <c r="D14" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E14" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>668</v>
+        <v>667</v>
+      </c>
+      <c r="G14" t="s">
+        <v>692</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -2759,24 +2810,24 @@
         <v>11</v>
       </c>
       <c r="D15" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E15" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="F15" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="G15" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="I15" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B16">
         <v>8</v>
@@ -2785,18 +2836,18 @@
         <v>12</v>
       </c>
       <c r="D16" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E16" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="F16" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -2805,18 +2856,18 @@
         <v>20</v>
       </c>
       <c r="D17" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E17" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="F17" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B18">
         <v>26</v>
@@ -2825,30 +2876,30 @@
         <v>52</v>
       </c>
       <c r="D18" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E18" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="F18" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="G18" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="H18" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="I18" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="J18" t="s">
-        <v>575</v>
-      </c>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B19">
         <v>4</v>
@@ -2857,21 +2908,21 @@
         <v>66</v>
       </c>
       <c r="D19" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E19" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="F19" t="s">
+        <v>628</v>
+      </c>
+      <c r="G19" t="s">
         <v>629</v>
       </c>
-      <c r="G19" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B20">
         <v>13</v>
@@ -2880,18 +2931,18 @@
         <v>29</v>
       </c>
       <c r="D20" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E20" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>631</v>
-      </c>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -2900,18 +2951,18 @@
         <v>5</v>
       </c>
       <c r="D21" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E21" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="F21" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B22">
         <v>1</v>
@@ -2920,12 +2971,12 @@
         <v>1</v>
       </c>
       <c r="D22" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.35">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B23">
         <v>16</v>
@@ -2934,15 +2985,15 @@
         <v>6</v>
       </c>
       <c r="D23" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E23" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.35">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B24">
         <v>2</v>
@@ -2951,18 +3002,18 @@
         <v>4</v>
       </c>
       <c r="D24" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E24" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F24" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.35">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B25">
         <v>85</v>
@@ -2971,48 +3022,51 @@
         <v>152</v>
       </c>
       <c r="D25" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E25" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F25" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="G25" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="H25" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="I25" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="J25" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="K25" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="L25" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="M25" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="N25" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="O25" s="1" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="P25" t="s">
-        <v>669</v>
-      </c>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.35">
+        <v>668</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B26">
         <v>0</v>
@@ -3021,12 +3075,12 @@
         <v>1</v>
       </c>
       <c r="D26" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.35">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B27">
         <v>0</v>
@@ -3035,12 +3089,12 @@
         <v>2</v>
       </c>
       <c r="D27" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.35">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B28">
         <v>0</v>
@@ -3049,12 +3103,12 @@
         <v>2</v>
       </c>
       <c r="D28" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.35">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B29">
         <v>3</v>
@@ -3063,21 +3117,21 @@
         <v>9</v>
       </c>
       <c r="D29" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E29" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F29" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="G29" t="s">
-        <v>494</v>
-      </c>
-    </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.35">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B30">
         <v>7</v>
@@ -3086,18 +3140,18 @@
         <v>12</v>
       </c>
       <c r="D30" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E30" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="F30" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.35">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B31">
         <v>1</v>
@@ -3106,12 +3160,12 @@
         <v>8</v>
       </c>
       <c r="D31" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.35">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B32">
         <v>19</v>
@@ -3120,27 +3174,27 @@
         <v>25</v>
       </c>
       <c r="D32" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E32" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="F32" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="G32" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="H32" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="I32" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B33">
         <v>0</v>
@@ -3149,15 +3203,15 @@
         <v>5</v>
       </c>
       <c r="D33" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E33" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B34">
         <v>5</v>
@@ -3166,33 +3220,33 @@
         <v>75</v>
       </c>
       <c r="D34" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E34" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F34" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="G34" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="H34" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="I34" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="J34" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="K34" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B35">
         <v>16</v>
@@ -3201,27 +3255,27 @@
         <v>51</v>
       </c>
       <c r="D35" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E35" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="F35" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="G35" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="I35" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="J35" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B36">
         <v>3</v>
@@ -3230,15 +3284,15 @@
         <v>1</v>
       </c>
       <c r="D36" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E36" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B37">
         <v>0</v>
@@ -3247,12 +3301,12 @@
         <v>13</v>
       </c>
       <c r="D37" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B38">
         <v>1</v>
@@ -3261,21 +3315,21 @@
         <v>4</v>
       </c>
       <c r="D38" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E38" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="F38" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="G38" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B39">
         <v>1</v>
@@ -3284,27 +3338,27 @@
         <v>6</v>
       </c>
       <c r="D39" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E39" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="F39" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="G39" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="H39" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="I39" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B40">
         <v>1</v>
@@ -3313,21 +3367,21 @@
         <v>45</v>
       </c>
       <c r="D40" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E40" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B41">
         <v>2</v>
@@ -3336,12 +3390,12 @@
         <v>3</v>
       </c>
       <c r="D41" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B42">
         <v>0</v>
@@ -3350,12 +3404,12 @@
         <v>1</v>
       </c>
       <c r="D42" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B43">
         <v>0</v>
@@ -3364,12 +3418,12 @@
         <v>1</v>
       </c>
       <c r="D43" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B44">
         <v>81</v>
@@ -3378,21 +3432,21 @@
         <v>144</v>
       </c>
       <c r="D44" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E44" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="F44" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="G44" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B45">
         <v>0</v>
@@ -3401,18 +3455,18 @@
         <v>3</v>
       </c>
       <c r="D45" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E45" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="F45" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B46">
         <v>1</v>
@@ -3421,33 +3475,33 @@
         <v>12</v>
       </c>
       <c r="D46" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E46" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="F46" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="G46" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="H46" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="I46" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="J46" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="K46" s="1" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B47">
         <v>47</v>
@@ -3456,24 +3510,24 @@
         <v>26</v>
       </c>
       <c r="D47" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E47" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="F47" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="G47" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="H47" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B48">
         <v>0</v>
@@ -3482,15 +3536,15 @@
         <v>3</v>
       </c>
       <c r="D48" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E48" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.35">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B49">
         <v>0</v>
@@ -3499,30 +3553,30 @@
         <v>15</v>
       </c>
       <c r="D49" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E49" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="F49" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="G49" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="H49" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="I49" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="J49" t="s">
-        <v>580</v>
-      </c>
-    </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.35">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B50">
         <v>0</v>
@@ -3531,18 +3585,18 @@
         <v>22</v>
       </c>
       <c r="D50" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E50" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="F50" t="s">
-        <v>636</v>
-      </c>
-    </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.35">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B51">
         <v>2</v>
@@ -3551,45 +3605,48 @@
         <v>13</v>
       </c>
       <c r="D51" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E51" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="F51" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="G51" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="H51" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="I51" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="J51" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="K51" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="L51" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="M51" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="N51" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="O51" t="s">
-        <v>619</v>
-      </c>
-    </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.35">
+        <v>618</v>
+      </c>
+      <c r="P51" t="s">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B52">
         <v>2</v>
@@ -3598,15 +3655,15 @@
         <v>4</v>
       </c>
       <c r="D52" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E52" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.35">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B53">
         <v>2</v>
@@ -3615,27 +3672,27 @@
         <v>17</v>
       </c>
       <c r="D53" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E53" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="F53" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="G53" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="H53" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="I53" t="s">
-        <v>638</v>
-      </c>
-    </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.35">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B54">
         <v>38</v>
@@ -3644,18 +3701,18 @@
         <v>20</v>
       </c>
       <c r="D54" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E54" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="F54" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.35">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="55" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B55">
         <v>0</v>
@@ -3664,18 +3721,18 @@
         <v>69</v>
       </c>
       <c r="D55" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E55" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>637</v>
-      </c>
-    </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.35">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B56">
         <v>0</v>
@@ -3684,15 +3741,15 @@
         <v>2</v>
       </c>
       <c r="D56" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="E56" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.35">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="57" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B57">
         <v>58</v>
@@ -3701,30 +3758,30 @@
         <v>51</v>
       </c>
       <c r="D57" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="E57" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="F57" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="G57" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="H57" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="I57" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="J57" t="s">
-        <v>582</v>
-      </c>
-    </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.35">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="58" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B58">
         <v>0</v>
@@ -3733,12 +3790,12 @@
         <v>62</v>
       </c>
       <c r="D58" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.35">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="59" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B59">
         <v>0</v>
@@ -3747,12 +3804,12 @@
         <v>1</v>
       </c>
       <c r="D59" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.35">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="60" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B60">
         <v>1</v>
@@ -3761,15 +3818,15 @@
         <v>4</v>
       </c>
       <c r="D60" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E60" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.35">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="61" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B61">
         <v>3</v>
@@ -3778,24 +3835,24 @@
         <v>19</v>
       </c>
       <c r="D61" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E61" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="F61" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="G61" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="H61" t="s">
-        <v>543</v>
-      </c>
-    </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.35">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="62" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B62">
         <v>0</v>
@@ -3804,12 +3861,12 @@
         <v>1</v>
       </c>
       <c r="D62" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.35">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="63" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B63">
         <v>11</v>
@@ -3818,18 +3875,18 @@
         <v>33</v>
       </c>
       <c r="D63" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E63" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="F63" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.35">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="64" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B64">
         <v>0</v>
@@ -3838,24 +3895,24 @@
         <v>29</v>
       </c>
       <c r="D64" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E64" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="F64" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="G64" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="H64" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B65">
         <v>0</v>
@@ -3864,12 +3921,12 @@
         <v>1</v>
       </c>
       <c r="D65" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B66">
         <v>21</v>
@@ -3878,21 +3935,21 @@
         <v>38</v>
       </c>
       <c r="D66" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E66" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="F66" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="G66" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B67">
         <v>0</v>
@@ -3901,18 +3958,18 @@
         <v>29</v>
       </c>
       <c r="D67" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E67" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="F67" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B68">
         <v>2</v>
@@ -3921,12 +3978,12 @@
         <v>0</v>
       </c>
       <c r="D68" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B69">
         <v>1</v>
@@ -3935,12 +3992,12 @@
         <v>0</v>
       </c>
       <c r="D69" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B70">
         <v>5</v>
@@ -3949,18 +4006,18 @@
         <v>5</v>
       </c>
       <c r="D70" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E70" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="F70" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B71">
         <v>1</v>
@@ -3969,12 +4026,12 @@
         <v>0</v>
       </c>
       <c r="D71" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B72">
         <v>8</v>
@@ -3983,21 +4040,21 @@
         <v>4</v>
       </c>
       <c r="D72" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E72" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="F72" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="G72" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B73">
         <v>1</v>
@@ -4006,12 +4063,12 @@
         <v>0</v>
       </c>
       <c r="D73" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B74">
         <v>0</v>
@@ -4020,12 +4077,12 @@
         <v>1</v>
       </c>
       <c r="D74" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B75">
         <v>1</v>
@@ -4034,15 +4091,15 @@
         <v>1</v>
       </c>
       <c r="D75" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E75" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B76">
         <v>1</v>
@@ -4051,12 +4108,12 @@
         <v>0</v>
       </c>
       <c r="D76" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B77">
         <v>10</v>
@@ -4065,27 +4122,27 @@
         <v>35</v>
       </c>
       <c r="D77" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E77" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="F77" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="G77" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="H77" s="1" t="s">
+        <v>643</v>
+      </c>
+      <c r="I77" s="1" t="s">
         <v>644</v>
-      </c>
-      <c r="I77" s="1" t="s">
-        <v>645</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B78">
         <v>1</v>
@@ -4094,18 +4151,18 @@
         <v>22</v>
       </c>
       <c r="D78" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E78" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="F78" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B79">
         <v>0</v>
@@ -4114,15 +4171,18 @@
         <v>34</v>
       </c>
       <c r="D79" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E79" t="s">
-        <v>368</v>
+        <v>367</v>
+      </c>
+      <c r="F79" t="s">
+        <v>677</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B80">
         <v>0</v>
@@ -4131,12 +4191,12 @@
         <v>40</v>
       </c>
       <c r="D80" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="81" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B81">
         <v>0</v>
@@ -4145,54 +4205,54 @@
         <v>19</v>
       </c>
       <c r="D81" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E81" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="F81" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="G81" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="H81" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="I81" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="J81" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="K81" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="L81" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="M81" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="N81" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="O81" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="P81" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="Q81" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="R81" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
     </row>
     <row r="82" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B82">
         <v>0</v>
@@ -4201,21 +4261,24 @@
         <v>34</v>
       </c>
       <c r="D82" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E82" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F82" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="G82" t="s">
-        <v>513</v>
+        <v>512</v>
+      </c>
+      <c r="H82" t="s">
+        <v>678</v>
       </c>
     </row>
     <row r="83" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B83">
         <v>0</v>
@@ -4224,12 +4287,12 @@
         <v>1</v>
       </c>
       <c r="D83" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="84" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B84">
         <v>10</v>
@@ -4238,18 +4301,18 @@
         <v>39</v>
       </c>
       <c r="D84" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E84" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="F84" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="85" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B85">
         <v>1</v>
@@ -4258,12 +4321,12 @@
         <v>0</v>
       </c>
       <c r="D85" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="86" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B86">
         <v>0</v>
@@ -4272,15 +4335,15 @@
         <v>79</v>
       </c>
       <c r="D86" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E86" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="87" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B87">
         <v>0</v>
@@ -4289,12 +4352,12 @@
         <v>2</v>
       </c>
       <c r="D87" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="88" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B88">
         <v>86</v>
@@ -4303,15 +4366,15 @@
         <v>1</v>
       </c>
       <c r="D88" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E88" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="89" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B89">
         <v>0</v>
@@ -4320,12 +4383,12 @@
         <v>3</v>
       </c>
       <c r="D89" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="90" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B90">
         <v>2</v>
@@ -4334,30 +4397,30 @@
         <v>39</v>
       </c>
       <c r="D90" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E90" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="F90" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="G90" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="H90" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="I90" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="J90" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="91" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B91">
         <v>0</v>
@@ -4366,18 +4429,18 @@
         <v>3</v>
       </c>
       <c r="D91" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E91" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="F91" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
     <row r="92" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B92">
         <v>0</v>
@@ -4386,43 +4449,40 @@
         <v>17</v>
       </c>
       <c r="D92" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E92" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="F92" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="G92" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="H92" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="I92" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="J92" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="K92" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="L92" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="M92" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="N92" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="O92" s="1" t="s">
-        <v>666</v>
-      </c>
-      <c r="P92" s="1" t="s">
-        <v>674</v>
+        <v>665</v>
       </c>
     </row>
     <row r="93" spans="1:18" x14ac:dyDescent="0.35">
@@ -4436,24 +4496,24 @@
         <v>92</v>
       </c>
       <c r="D93" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E93" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="F93" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="G93" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="H93" s="1" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
     </row>
     <row r="94" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B94">
         <v>0</v>
@@ -4462,15 +4522,15 @@
         <v>48</v>
       </c>
       <c r="D94" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E94" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="95" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B95">
         <v>0</v>
@@ -4479,21 +4539,21 @@
         <v>15</v>
       </c>
       <c r="D95" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E95" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="F95" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="G95" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
     </row>
     <row r="96" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B96">
         <v>7</v>
@@ -4502,21 +4562,21 @@
         <v>10</v>
       </c>
       <c r="D96" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E96" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F96" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="G96" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B97">
         <v>18</v>
@@ -4525,21 +4585,21 @@
         <v>31</v>
       </c>
       <c r="D97" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E97" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="F97" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="G97" s="1" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B98">
         <v>15</v>
@@ -4548,30 +4608,30 @@
         <v>3</v>
       </c>
       <c r="D98" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E98" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="F98" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="G98" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="H98" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="I98" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="J98" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B99">
         <v>16</v>
@@ -4580,24 +4640,27 @@
         <v>39</v>
       </c>
       <c r="D99" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E99" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="F99" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="G99" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="H99" t="s">
-        <v>549</v>
+        <v>548</v>
+      </c>
+      <c r="I99" t="s">
+        <v>682</v>
       </c>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B100">
         <v>0</v>
@@ -4606,21 +4669,21 @@
         <v>39</v>
       </c>
       <c r="D100" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E100" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="F100" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="G100" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B101">
         <v>14</v>
@@ -4629,30 +4692,30 @@
         <v>45</v>
       </c>
       <c r="D101" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E101" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="F101" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="G101" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="H101" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="I101" s="1" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="J101" s="1" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B102">
         <v>0</v>
@@ -4661,18 +4724,18 @@
         <v>3</v>
       </c>
       <c r="D102" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E102" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="F102" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B103">
         <v>0</v>
@@ -4681,12 +4744,12 @@
         <v>1</v>
       </c>
       <c r="D103" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B104">
         <v>1</v>
@@ -4695,12 +4758,12 @@
         <v>1</v>
       </c>
       <c r="D104" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B105">
         <v>1</v>
@@ -4709,12 +4772,12 @@
         <v>0</v>
       </c>
       <c r="D105" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B106">
         <v>0</v>
@@ -4723,18 +4786,18 @@
         <v>87</v>
       </c>
       <c r="D106" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E106" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="F106" s="1" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B107">
         <v>0</v>
@@ -4743,12 +4806,12 @@
         <v>1</v>
       </c>
       <c r="D107" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B108">
         <v>3</v>
@@ -4757,12 +4820,12 @@
         <v>4</v>
       </c>
       <c r="D108" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B109">
         <v>0</v>
@@ -4771,12 +4834,12 @@
         <v>1</v>
       </c>
       <c r="D109" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A110" s="1" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="B110">
         <v>1</v>
@@ -4785,15 +4848,15 @@
         <v>0</v>
       </c>
       <c r="D110" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E110" s="1" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
     </row>
     <row r="111" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B111">
         <v>25</v>
@@ -4802,18 +4865,18 @@
         <v>28</v>
       </c>
       <c r="D111" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E111" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F111" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B112">
         <v>0</v>
@@ -4822,18 +4885,18 @@
         <v>2</v>
       </c>
       <c r="D112" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E112" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="F112" t="s">
-        <v>657</v>
-      </c>
-    </row>
-    <row r="113" spans="1:15" x14ac:dyDescent="0.35">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="113" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B113">
         <v>42</v>
@@ -4842,39 +4905,45 @@
         <v>0</v>
       </c>
       <c r="D113" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="E113" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="F113" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="G113" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="H113" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="I113" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="J113" t="s">
+        <v>653</v>
+      </c>
+      <c r="K113" t="s">
+        <v>389</v>
+      </c>
+      <c r="L113" t="s">
         <v>654</v>
       </c>
-      <c r="K113" t="s">
-        <v>390</v>
-      </c>
-      <c r="L113" t="s">
-        <v>655</v>
-      </c>
       <c r="M113" t="s">
-        <v>677</v>
-      </c>
-    </row>
-    <row r="114" spans="1:15" x14ac:dyDescent="0.35">
+        <v>676</v>
+      </c>
+      <c r="N113" t="s">
+        <v>684</v>
+      </c>
+      <c r="O113" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="114" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B114">
         <v>3</v>
@@ -4883,12 +4952,12 @@
         <v>1</v>
       </c>
       <c r="D114" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="115" spans="1:15" x14ac:dyDescent="0.35">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="115" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B115">
         <v>123</v>
@@ -4897,15 +4966,15 @@
         <v>118</v>
       </c>
       <c r="D115" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E115" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="116" spans="1:15" x14ac:dyDescent="0.35">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="116" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B116">
         <v>26</v>
@@ -4914,24 +4983,33 @@
         <v>11</v>
       </c>
       <c r="D116" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="E116" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F116" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="G116" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="H116" s="1" t="s">
-        <v>651</v>
-      </c>
-    </row>
-    <row r="117" spans="1:15" x14ac:dyDescent="0.35">
+        <v>650</v>
+      </c>
+      <c r="I116" s="1" t="s">
+        <v>673</v>
+      </c>
+      <c r="J116" t="s">
+        <v>683</v>
+      </c>
+      <c r="K116" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="117" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B117">
         <v>0</v>
@@ -4940,18 +5018,18 @@
         <v>9</v>
       </c>
       <c r="D117" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E117" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="F117" t="s">
-        <v>474</v>
-      </c>
-    </row>
-    <row r="118" spans="1:15" x14ac:dyDescent="0.35">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="118" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B118">
         <v>0</v>
@@ -4960,18 +5038,18 @@
         <v>4</v>
       </c>
       <c r="D118" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E118" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F118" t="s">
-        <v>475</v>
-      </c>
-    </row>
-    <row r="119" spans="1:15" x14ac:dyDescent="0.35">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="119" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B119">
         <v>0</v>
@@ -4980,42 +5058,42 @@
         <v>16</v>
       </c>
       <c r="D119" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E119" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F119" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="G119" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="H119" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="I119" t="s">
+        <v>647</v>
+      </c>
+      <c r="J119" t="s">
+        <v>586</v>
+      </c>
+      <c r="K119" t="s">
+        <v>595</v>
+      </c>
+      <c r="L119" t="s">
+        <v>602</v>
+      </c>
+      <c r="M119" t="s">
+        <v>609</v>
+      </c>
+      <c r="N119" t="s">
         <v>648</v>
       </c>
-      <c r="J119" t="s">
-        <v>587</v>
-      </c>
-      <c r="K119" t="s">
-        <v>596</v>
-      </c>
-      <c r="L119" t="s">
-        <v>603</v>
-      </c>
-      <c r="M119" t="s">
-        <v>610</v>
-      </c>
-      <c r="N119" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="120" spans="1:15" x14ac:dyDescent="0.35">
+    </row>
+    <row r="120" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B120">
         <v>4</v>
@@ -5024,15 +5102,15 @@
         <v>1</v>
       </c>
       <c r="D120" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="E120" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="121" spans="1:15" x14ac:dyDescent="0.35">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="121" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A121" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B121">
         <v>7</v>
@@ -5041,45 +5119,48 @@
         <v>73</v>
       </c>
       <c r="D121" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E121" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="F121" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="G121" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H121" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="I121" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="J121" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="K121" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="L121" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="M121" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="N121" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="O121" t="s">
-        <v>642</v>
-      </c>
-    </row>
-    <row r="122" spans="1:15" x14ac:dyDescent="0.35">
+        <v>641</v>
+      </c>
+      <c r="P121" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="122" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B122">
         <v>1</v>
@@ -5088,12 +5169,12 @@
         <v>0</v>
       </c>
       <c r="D122" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="123" spans="1:15" x14ac:dyDescent="0.35">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="123" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B123">
         <v>11</v>
@@ -5102,15 +5183,15 @@
         <v>2</v>
       </c>
       <c r="D123" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E123" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="124" spans="1:15" x14ac:dyDescent="0.35">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="124" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B124">
         <v>0</v>
@@ -5119,30 +5200,30 @@
         <v>132</v>
       </c>
       <c r="D124" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E124" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="F124" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="G124" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="H124" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="I124" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="J124" t="s">
-        <v>589</v>
-      </c>
-    </row>
-    <row r="125" spans="1:15" x14ac:dyDescent="0.35">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="125" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B125">
         <v>0</v>
@@ -5151,18 +5232,18 @@
         <v>4</v>
       </c>
       <c r="D125" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E125" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="F125" t="s">
-        <v>659</v>
-      </c>
-    </row>
-    <row r="126" spans="1:15" x14ac:dyDescent="0.35">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="126" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B126">
         <v>4</v>
@@ -5171,24 +5252,24 @@
         <v>53</v>
       </c>
       <c r="D126" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E126" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="F126" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="G126" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="H126" t="s">
-        <v>555</v>
-      </c>
-    </row>
-    <row r="127" spans="1:15" x14ac:dyDescent="0.35">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="127" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B127">
         <v>0</v>
@@ -5197,12 +5278,12 @@
         <v>7</v>
       </c>
       <c r="D127" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="128" spans="1:15" x14ac:dyDescent="0.35">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="128" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B128">
         <v>0</v>
@@ -5211,15 +5292,15 @@
         <v>1</v>
       </c>
       <c r="D128" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E128" t="s">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.35">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="129" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B129">
         <v>14</v>
@@ -5228,15 +5309,15 @@
         <v>32</v>
       </c>
       <c r="D129" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E129" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.35">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="130" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B130">
         <v>0</v>
@@ -5245,15 +5326,15 @@
         <v>16</v>
       </c>
       <c r="D130" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E130" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.35">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="131" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B131">
         <v>2</v>
@@ -5262,15 +5343,15 @@
         <v>16</v>
       </c>
       <c r="D131" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E131" t="s">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.35">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="132" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B132">
         <v>2</v>
@@ -5279,12 +5360,12 @@
         <v>5</v>
       </c>
       <c r="D132" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.35">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="133" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B133">
         <v>21</v>
@@ -5293,18 +5374,18 @@
         <v>3</v>
       </c>
       <c r="D133" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E133" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="F133" t="s">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.35">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="134" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B134">
         <v>0</v>
@@ -5313,18 +5394,18 @@
         <v>32</v>
       </c>
       <c r="D134" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E134" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="F134" t="s">
-        <v>481</v>
-      </c>
-    </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.35">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="135" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B135">
         <v>88</v>
@@ -5333,15 +5414,15 @@
         <v>0</v>
       </c>
       <c r="D135" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E135" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.35">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="136" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B136">
         <v>2</v>
@@ -5350,12 +5431,12 @@
         <v>0</v>
       </c>
       <c r="D136" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.35">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="137" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B137">
         <v>1</v>
@@ -5364,12 +5445,12 @@
         <v>0</v>
       </c>
       <c r="D137" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.35">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="138" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B138">
         <v>43</v>
@@ -5378,18 +5459,18 @@
         <v>0</v>
       </c>
       <c r="D138" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E138" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="F138" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.35">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="139" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B139">
         <v>0</v>
@@ -5398,12 +5479,12 @@
         <v>1</v>
       </c>
       <c r="D139" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.35">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="140" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B140">
         <v>4</v>
@@ -5412,15 +5493,15 @@
         <v>0</v>
       </c>
       <c r="D140" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E140" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.35">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="141" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B141">
         <v>1</v>
@@ -5429,12 +5510,12 @@
         <v>0</v>
       </c>
       <c r="D141" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="142" spans="1:10" x14ac:dyDescent="0.35">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="142" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B142">
         <v>79</v>
@@ -5443,21 +5524,21 @@
         <v>5</v>
       </c>
       <c r="D142" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E142" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F142" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="G142" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.35">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="143" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B143">
         <v>22</v>
@@ -5466,30 +5547,36 @@
         <v>0</v>
       </c>
       <c r="D143" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E143" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F143" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="G143" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="H143" t="s">
+        <v>660</v>
+      </c>
+      <c r="I143" t="s">
         <v>661</v>
       </c>
-      <c r="I143" t="s">
+      <c r="J143" t="s">
         <v>662</v>
       </c>
-      <c r="J143" t="s">
-        <v>663</v>
-      </c>
-    </row>
-    <row r="144" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K143" t="s">
+        <v>690</v>
+      </c>
+      <c r="L143" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="144" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B144">
         <v>2</v>
@@ -5498,18 +5585,18 @@
         <v>3</v>
       </c>
       <c r="D144" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="E144" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="F144" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
     </row>
     <row r="145" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B145">
         <v>3</v>
@@ -5518,24 +5605,24 @@
         <v>16</v>
       </c>
       <c r="D145" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="E145" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="F145" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="G145" s="1" t="s">
+        <v>626</v>
+      </c>
+      <c r="H145" s="1" t="s">
         <v>627</v>
-      </c>
-      <c r="H145" s="1" t="s">
-        <v>628</v>
       </c>
     </row>
     <row r="146" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B146">
         <v>5</v>
@@ -5544,15 +5631,15 @@
         <v>29</v>
       </c>
       <c r="D146" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="E146" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="147" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A147" s="1" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="B147">
         <v>1</v>
@@ -5561,18 +5648,21 @@
         <v>0</v>
       </c>
       <c r="D147" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="E147" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="F147" t="s">
-        <v>671</v>
+        <v>670</v>
+      </c>
+      <c r="G147" t="s">
+        <v>689</v>
       </c>
     </row>
     <row r="148" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B148">
         <v>0</v>
@@ -5581,12 +5671,12 @@
         <v>1</v>
       </c>
       <c r="D148" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="149" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B149">
         <v>0</v>
@@ -5595,12 +5685,12 @@
         <v>1</v>
       </c>
       <c r="D149" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="150" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B150">
         <v>0</v>
@@ -5609,12 +5699,12 @@
         <v>2</v>
       </c>
       <c r="D150" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="151" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B151">
         <v>0</v>
@@ -5623,12 +5713,12 @@
         <v>13</v>
       </c>
       <c r="D151" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="152" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B152">
         <v>15</v>
@@ -5637,18 +5727,18 @@
         <v>34</v>
       </c>
       <c r="D152" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E152" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F152" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
     </row>
     <row r="153" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B153">
         <v>2</v>
@@ -5657,18 +5747,18 @@
         <v>5</v>
       </c>
       <c r="D153" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E153" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="F153" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="154" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B154">
         <v>0</v>
@@ -5677,18 +5767,18 @@
         <v>4</v>
       </c>
       <c r="D154" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E154" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="F154" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="155" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B155">
         <v>0</v>
@@ -5697,15 +5787,15 @@
         <v>2</v>
       </c>
       <c r="D155" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E155" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="156" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B156">
         <v>0</v>
@@ -5714,12 +5804,12 @@
         <v>1</v>
       </c>
       <c r="D156" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="157" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B157">
         <v>49</v>
@@ -5728,24 +5818,24 @@
         <v>91</v>
       </c>
       <c r="D157" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E157" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="F157" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="G157" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="H157" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
     </row>
     <row r="158" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B158">
         <v>0</v>
@@ -5754,12 +5844,12 @@
         <v>1</v>
       </c>
       <c r="D158" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="159" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="B159">
         <v>0</v>
@@ -5768,26 +5858,26 @@
         <v>0</v>
       </c>
       <c r="D159" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
     </row>
     <row r="160" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A160" s="1" t="s">
+        <v>663</v>
+      </c>
+      <c r="B160">
+        <v>0</v>
+      </c>
+      <c r="C160">
+        <v>0</v>
+      </c>
+      <c r="D160" s="1" t="s">
         <v>664</v>
-      </c>
-      <c r="B160">
-        <v>0</v>
-      </c>
-      <c r="C160">
-        <v>0</v>
-      </c>
-      <c r="D160" s="1" t="s">
-        <v>665</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A161" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B161">
         <v>0</v>
@@ -5796,7 +5886,7 @@
         <v>0</v>
       </c>
       <c r="D161" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
     </row>
   </sheetData>

</xml_diff>